<commit_message>
docs: analyze developer stakeholder
</commit_message>
<xml_diff>
--- a/docs/analysis.v1.xlsx
+++ b/docs/analysis.v1.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binhld\Desktop\GameStore\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463230BF-7644-4F98-A6D5-3AF31589B06C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6815A571-8B17-49B3-817F-23A69DF38924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37710" windowHeight="21840" activeTab="1" xr2:uid="{AD2317E5-E67D-422E-8F1C-062DBE876A8A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37710" windowHeight="21840" xr2:uid="{AD2317E5-E67D-422E-8F1C-062DBE876A8A}"/>
   </bookViews>
   <sheets>
-    <sheet name="overal" sheetId="1" r:id="rId1"/>
-    <sheet name="end_users" sheetId="2" r:id="rId2"/>
+    <sheet name="version" sheetId="4" r:id="rId1"/>
+    <sheet name="overview" sheetId="1" r:id="rId2"/>
+    <sheet name="end_users" sheetId="2" r:id="rId3"/>
+    <sheet name="developers" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="165">
   <si>
     <t>Role:
 You are a senior business analyst with deep knowledge of the PC game distribution ecosystem.
@@ -115,12 +117,6 @@
     <t>Developer Relation</t>
   </si>
   <si>
-    <t>Trust &amp; safety</t>
-  </si>
-  <si>
-    <t>Fraud, refund, moderation</t>
-  </si>
-  <si>
     <t>Curation onboarding, featuring, sales events</t>
   </si>
   <si>
@@ -537,6 +533,619 @@
   </si>
   <si>
     <t>3. Game Publishers</t>
+  </si>
+  <si>
+    <t>Context: Early phase of designing a new Video Game Distribution Platforms.  There are 5 categories of stakeholder involve in the system: Gamers/End Users; Game Developers/Game Studios; Game Publishers; Content Creators &amp; Influencers/Affiliates; Payment Providers
+Tasks:
+* Compare platform features for Game Developers / Game Stuios stakeholder
+* Explain how this stakeholder interact with the system (explain in a simple worflow diagram)
+Output requirements:
+* Use clear, simple language.
+* Be specific and structured.
+* Use tables where helpful.
+* Provide real-world examples to illustrate workflows or interactions.
+* Highlight differences between Steam and Epic when relevant.
+* Focus on practical, real industry practices (not theory).</t>
+  </si>
+  <si>
+    <t>Developers / Studios Goals</t>
+  </si>
+  <si>
+    <t>Developers / Studios typically want to:
+- Reduce development effort
+- Reduce operational effort
+- Receive analytics data</t>
+  </si>
+  <si>
+    <t>Trust &amp; Safety</t>
+  </si>
+  <si>
+    <t>Fraud, refund, moderation, tax, policies</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Manage Builds &amp; Updates:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> For shipping patches, new contents</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Game Monitoring: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>For knowing game performance, crash reports, player metrics</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Publishing Access:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> For submit and deliver the game</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Developer Tools &amp; SDK: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Provide platform services: users, achivements, cloud saves, anti-cheat, matchmaking</t>
+    </r>
+  </si>
+  <si>
+    <t>v1</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>v1.1</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Account and Social</t>
+  </si>
+  <si>
+    <t>Multiplayer</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Stats:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Define the stats for your game in the Developer Portal. You can include any statistical data about a player that you want to track, for example the number of items the player has collected. You can use these stats to determine when to unlock achievements and how to rank players in leaderboards.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">- Leaderboards: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Define leaderboards for your game, choose the stats to include, how you rank players, and the lifespan of the leaderboards.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Achievements:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Access data about player achievements, unlock them for a player, get data on a player's progression for an achievement, and send notifications to players when they unlock an achievement.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Player Data Storage:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Save, download, copy, and delete player-related data for your game on cloud servers in encrypted form
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Metrics:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Set up the game analytics dashboard in the Developer Portal and track worldwide game activity, player retention, and online player counts. You can view your game’s usage data, including players’ active sessions and past sessions</t>
+    </r>
+  </si>
+  <si>
+    <t>Player and Game Data</t>
+  </si>
+  <si>
+    <t>Trust and Safety</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Authentication:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Authenticate players, get authorization credentials (access tokens)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- User Info:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Obtain player information, such as their name or avatar
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Friends:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Enable player to invite their friends to join a game-play session
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Presense:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Display a player's status (online, offline, playing) in a game</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Anti-Cheat:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Prevent and detect players cheating within your game
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Reports:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Collect and publish player behavior to player reports. View details about player cheating, verbal abuse and offensive profiles
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Sanctions:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Define and manage sanctions for your game. In the Developer Portal, you can view the details of all sanctions placed on a player</t>
+    </r>
+  </si>
+  <si>
+    <t>add: overview + end_users</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Peer-to-Peer (P2P):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Enable players to connect with other players in a game
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Lobbies:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Enable players to create, join, leave and remove lobbies
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Sessions:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Allow player to host, find, and interact with online gaming sessions
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Communication:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Allow player to create and manage voice chat/text chat room during matches or in lobbies</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Developer Tools &amp; SDK APIs</t>
+  </si>
+  <si>
+    <t>Account Registration</t>
+  </si>
+  <si>
+    <t>Company Verification</t>
+  </si>
+  <si>
+    <t>Legal Agreements</t>
+  </si>
+  <si>
+    <t>Tax and Financial setup</t>
+  </si>
+  <si>
+    <t>Country tax compliance, payment setup</t>
+  </si>
+  <si>
+    <t>Developer Portal Access</t>
+  </si>
+  <si>
+    <t>Developer request to create an account by providing information such as name, website, email, etc</t>
+  </si>
+  <si>
+    <t>Platform verify identity to prevent fraud and privacy</t>
+  </si>
+  <si>
+    <t>Developer sign a contract with platform by agree to platform terms&amp;conditions</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Developer Onboarding: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>For registering a new</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>developer account</t>
+    </r>
+  </si>
+  <si>
+    <t>2. Developer Onboarding</t>
+  </si>
+  <si>
+    <t>3. Publishing A New Game</t>
+  </si>
+  <si>
+    <t>Game Project Creation</t>
+  </si>
+  <si>
+    <t>Create a new game project with basic information such as title, genre, platform, etc</t>
+  </si>
+  <si>
+    <t>Store Page Management</t>
+  </si>
+  <si>
+    <t>Configure in detail how the game appear in the store front: gameplay, screeshots, trailers, system requirements, etc</t>
+  </si>
+  <si>
+    <t>Game Build</t>
+  </si>
+  <si>
+    <t>Developer upload actual playable game files</t>
+  </si>
+  <si>
+    <t>Developer configure gameplay-related platform features: achivements, clould saves, items, etc</t>
+  </si>
+  <si>
+    <t>Pricing Settings</t>
+  </si>
+  <si>
+    <t>Distribution Settings</t>
+  </si>
+  <si>
+    <t>Publisher configure base price (price in main currency), regional pricing (auto or manual)</t>
+  </si>
+  <si>
+    <t>Developer gain access to the portal, where they can submit a new game</t>
+  </si>
+  <si>
+    <t>Gameplay Settings</t>
+  </si>
+  <si>
+    <t>Review Compliance</t>
+  </si>
+  <si>
+    <t>Platform check if the game pass all compliance checklist: content, age rating, build quality check, etc</t>
+  </si>
+  <si>
+    <t>Publisher configure distribution region, release date, early access date for tester (test build, preview store page)</t>
+  </si>
+  <si>
+    <t>Publish</t>
+  </si>
+  <si>
+    <t>Lauch button or scheduled lauch</t>
+  </si>
+  <si>
+    <t>add: developers (NOT FINISHED YET)</t>
   </si>
 </sst>
 </file>
@@ -594,7 +1203,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -604,6 +1213,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -635,7 +1250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -659,20 +1274,51 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1006,6 +1652,53 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1625A7DC-D869-4959-A362-A8167AA73A61}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="15.7109375" style="15" customWidth="1"/>
+    <col min="3" max="3" width="33.42578125" style="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="19">
+        <v>46054</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="22">
+        <v>46082</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{666A3806-41B2-4590-B8D6-460ACACFC314}">
   <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1023,14 +1716,14 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="B3" s="13"/>
-    </row>
-    <row r="4" spans="1:2" s="15" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="14"/>
-      <c r="B4" s="14"/>
+      <c r="A3" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="27"/>
+    </row>
+    <row r="4" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
@@ -1058,7 +1751,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>4</v>
@@ -1109,7 +1802,7 @@
         <v>18</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -1117,15 +1810,15 @@
         <v>19</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>21</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1136,9 +1829,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B87DD229-A2A4-421F-A907-46D1FB9E2C23}">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.140625" bestFit="1" customWidth="1"/>
@@ -1151,67 +1844,67 @@
         <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-    </row>
-    <row r="4" spans="1:3" s="18" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-    </row>
-    <row r="5" spans="1:3" s="18" customFormat="1" ht="106.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+    </row>
+    <row r="5" spans="1:3" ht="106.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" s="17"/>
+        <v>86</v>
+      </c>
+      <c r="C5" s="14"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1219,201 +1912,210 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C26" s="4"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C28" s="4"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C30" s="4"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="4"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B37" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C37" s="4"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C38" s="4"/>
     </row>
@@ -1421,82 +2123,82 @@
       <c r="A39" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C39" s="4"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
-        <v>49</v>
+      <c r="A42" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>66</v>
-      </c>
+      <c r="A43" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" s="4"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B44" s="10" t="s">
-        <v>110</v>
+        <v>49</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="C44" s="4"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C45" s="4"/>
+        <v>50</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B46" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>75</v>
-      </c>
+      <c r="C46" s="4"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C47" s="4"/>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>54</v>
       </c>
       <c r="C48" s="4"/>
     </row>
@@ -1505,125 +2207,397 @@
         <v>56</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C49" s="4"/>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="2" t="s">
-        <v>106</v>
+      <c r="A52" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B53" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>66</v>
-      </c>
+      <c r="A53" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C53" s="4"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C54" s="4"/>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>60</v>
+        <v>105</v>
+      </c>
+      <c r="B55" s="12" t="s">
+        <v>106</v>
       </c>
       <c r="C55" s="4"/>
     </row>
     <row r="56" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B56" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C56" s="4"/>
-    </row>
-    <row r="57" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B57" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>71</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C57" s="4"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C58" s="4"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B59" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C59" s="4"/>
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>76</v>
+        <v>62</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:C3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94723F64-BC22-49F8-B5F9-24B03B3E0BB2}">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="A1:C36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="102.5703125" customWidth="1"/>
+    <col min="3" max="3" width="7.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="225" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+      <c r="A3" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+    </row>
+    <row r="4" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+    </row>
+    <row r="5" spans="1:3" ht="61.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="14"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B61" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B62" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>81</v>
-      </c>
+    </row>
+    <row r="14" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:3" ht="180" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" s="4"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C21" s="4"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C22" s="4"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C23" s="4"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24" s="4"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C25" s="4"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" s="4"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C30" s="4"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C31" s="4"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" s="4"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C36" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>